<commit_message>
투자 대시보드 2026-10-16 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-15.xlsx
+++ b/technicals/exports/2026-10-15.xlsx
@@ -142,7 +142,7 @@
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 의약품과 치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
+          <ns0:t>전 세계에서 의약품·치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
@@ -221,7 +221,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 시설 유지관리, 엔지니어링 및 인프라 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 시설 유지관리·엔지니어링·인프라 솔루션을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -300,7 +300,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>중고차 판매·구매 딜러를 연결해 실시간 기업 간 거래를 지원하는 디지털 도매 경매 플랫폼 기업.</ns0:t>
+          <ns0:t>중고차 판매·구매 딜러 간 실시간 거래를 지원하는 디지털 도매 경매 플랫폼 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -379,7 +379,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 클라우드 기반 인적자본관리 플랫폼과 인사 업무 아웃소싱 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>전 세계에 클라우드 기반 인적자본관리 플랫폼과 인사 업무 아웃소싱을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -458,7 +458,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 단독주택·콘도 소유자와 빈 주택 등을 위한 주거용 부동산 보험을 제공.</ns0:t>
+          <ns0:t>미국에서 단독주택·콘도·빈 주택 등을 위한 주거용 부동산 보험 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
@@ -616,7 +616,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 남성·여성·아동용 의류, 개인관리 제품, 액세서리를 판매하는 온·오프라인 소매기업.</ns0:t>
+          <ns0:t>전 세계에서 남성·여성·아동 의류와 개인관리 제품·액세서리를 판매하는 온·오프라인 소매기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -695,7 +695,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 사격 스포츠 액세서리, 칼 등 야외활동 제품과 용품을 제공하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 사격 스포츠 액세서리·칼 등 야외활동 제품과 용품을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -774,7 +774,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 의료기관·연구기관 등에 의료용품, 의료기기, 실험실 장비 및 진단 제품을 개발·제조·판매.</ns0:t>
+          <ns0:t>전 세계 의료·연구기관 등에 의료용품·의료기기·실험실 장비·진단 제품을 개발·제조·판매하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -853,7 +853,7 @@
       </ns0:c>
       <ns0:c r="F11" t="inlineStr">
         <ns0:is>
-          <ns0:t>다발성경화증, 척수성 근위축증 등 치료제를 연구·개발·제조·공급하는 기업.</ns0:t>
+          <ns0:t>다발성경화증·척수성 근위축증 등 치료제를 연구·개발·제조·공급하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G11">
@@ -932,7 +932,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 동부 지역에서 식료품·신선식품·일반상품·휘발유 등을 판매하는 회원제 창고형 매장 운영기업.</ns0:t>
+          <ns0:t>미국 동부에서 식료품·신선식품·일반상품·휘발유 등을 판매하는 회원제 창고형 매장 운영기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1011,7 +1011,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>다양한 규모의 조직이 장소와 기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
+          <ns0:t>다양한 규모의 조직이 장소·기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1090,7 +1090,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 석유·가스 사업을 운영하며 가스·저탄소 에너지, 석유 생산 및 고객·제품 부문을 영위.</ns0:t>
+          <ns0:t>전 세계에서 가스·저탄소 에너지, 석유 생산, 고객·제품 부문 등 석유·가스 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1169,7 +1169,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 금융서비스·기술·바이오·제약 등의 기업과 합병·인수 등 사업결합을 추진하는 기업.</ns0:t>
+          <ns0:t>주요 영업활동 없이 금융서비스·기술·바이오·제약 기업 등과 합병·인수 등 사업결합을 추진하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1245,7 +1245,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료기술 기업으로 급성기 환자용 현장 뇌파검사 플랫폼인 Ceribell System을 개발.</ns0:t>
+          <ns0:t>급성기 환자용 현장 뇌파검사 플랫폼 Ceribell System을 개발하는 미국 의료기술 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1403,7 +1403,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업 활동 없이 합병, 주식 교환, 자산 인수, 자본 재편 등 기업 결합을 추진.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수·자본 재편 등 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1479,7 +1479,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>고급 장기체류 호텔과 프리미엄 브랜드의 선택형 서비스 호텔에 주로 투자하는 상장 부동산투자신탁.</ns0:t>
+          <ns0:t>고급 장기체류 호텔과 프리미엄 브랜드 선택형 서비스 호텔에 주로 투자하는 상장 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1558,7 +1558,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 보험 보장이 부족한 가정과 기업에 프로그램·서비스를 제공하는 관리형 의료 기업.</ns0:t>
+          <ns0:t>미국 내 보험 보장이 부족한 가정·기업에 프로그램과 서비스를 제공하는 관리형 의료 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1716,7 +1716,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소 등을 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
+          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소를 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1795,7 +1795,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매하는 기업.</ns0:t>
+          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1953,7 +1953,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>AI 등 기술을 활용해 산재보상·일반 및 자동차 배상책임 관리와 병원비 심사·지급 적정성 솔루션을 제공.</ns0:t>
+          <ns0:t>AI 등을 활용해 산재보상·일반 및 자동차 배상책임 관리, 병원비 심사·지급 적정성 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2032,7 +2032,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·천연가스 탐사, 개발, 생산, 운송 등을 포함한 통합 에너지 및 화학 사업을 영위.</ns0:t>
+          <ns0:t>원유·천연가스 탐사·개발·생산·운송 등을 포함한 통합 에너지·화학 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2190,7 +2190,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국·중국·독일 등 전 세계에서 구매자와 판매자를 연결하는 온라인 마켓플레이스 운영기업.</ns0:t>
+          <ns0:t>미국·영국·중국·독일 등 전 세계 구매자와 판매자를 연결하는 온라인 마켓플레이스 운영기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2348,7 +2348,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 구매자와 판매자를 연결하는 Etsy·Depop 온라인 마켓플레이스를 운영하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 구매자와 판매자를 연결하는 Etsy·Depop 온라인 마켓플레이스 운영기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2651,7 +2651,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>개인·소기업·기업 고객에게 은행·신탁·금융 서비스를 제공하는 은행을 보유한 지주회사.</ns0:t>
+          <ns0:t>개인·소기업·기업에 은행·신탁·금융 서비스를 제공하는 은행을 보유한 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2730,7 +2730,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 의료용 의류, 신발 등 생활용품을 소비자에게 직접 판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 의료용 의류·신발 등 생활용품을 소비자에게 직접 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2809,7 +2809,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>증권 중개·매매, 시장조성, 투자 리서치·자문, 소매·상업은행 및 보험 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>증권 중개·매매·시장조성·투자 리서치·자문과 소매·상업은행 및 보험 서비스를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2888,7 +2888,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 고객 경험과 직원 경험을 위한 서비스형 소프트웨어를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 고객·직원 경험을 위한 서비스형 소프트웨어를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -3125,7 +3125,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·유럽 등에서 미충족 의료 수요 분야의 의약품과 HIV-1 치료제를 발굴·개발·상용화하는 바이오제약사.</ns0:t>
+          <ns0:t>미국·유럽 등에서 미충족 의료 수요 분야 의약품과 HIV-1 치료제를 발굴·개발·상용화하는 바이오제약사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3204,7 +3204,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임, 수집품, 엔터테인먼트 제품을 판매하는 기업.</ns0:t>
+          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임·수집품·엔터테인먼트 제품을 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3283,7 +3283,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 및 해외에서 에너지 서비스를 제공하며 전력·천연가스 재판매와 재생에너지 사업을 영위.</ns0:t>
+          <ns0:t>미국 및 해외에서 전력·천연가스 재판매와 재생에너지 등 에너지 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3362,7 +3362,7 @@
       </ns0:c>
       <ns0:c r="F43" t="inlineStr">
         <ns0:is>
-          <ns0:t>독자 효소와 기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
+          <ns0:t>독자 효소·기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G43">
@@ -3441,7 +3441,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험을 제공하며 보험·마켓플레이스 부문을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험과 마켓플레이스 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3520,7 +3520,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3599,7 +3599,7 @@
       </ns0:c>
       <ns0:c r="F46" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G46">
@@ -3678,7 +3678,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 개인 및 상업용 주거용 부동산 보험을 제공.</ns0:t>
+          <ns0:t>자회사를 통해 개인 및 상업용 주거용 부동산 보험을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3757,7 +3757,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>하나 이상의 기업과 합병·주식교환·자산인수 등 기업결합을 추진하는 기업.</ns0:t>
+          <ns0:t>하나 이상의 기업과 합병·주식교환·자산인수 등 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3833,7 +3833,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공하는 기업.</ns0:t>
+          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -3912,7 +3912,7 @@
       </ns0:c>
       <ns0:c r="F50" t="inlineStr">
         <ns0:is>
-          <ns0:t>식품·음료·건강 및 바이오과학·향료와 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
+          <ns0:t>식품·음료·건강·바이오과학·향료 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G50">
@@ -3991,7 +3991,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다에서 주입 펌프와 관련 제품·서비스를 제공하며 환자 서비스와 의료기기 솔루션을 운영.</ns0:t>
+          <ns0:t>미국·캐나다에서 주입 펌프와 관련 제품·서비스, 환자 서비스 및 의료기기 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4070,7 +4070,7 @@
       </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 장난감, 소비재·전자제품, 아동용 가구, 의상, 스포츠용품, 가정용 가구 등을 제작·판매.</ns0:t>
+          <ns0:t>전 세계에서 장난감, 소비재·전자제품, 아동·가정용 가구, 의상, 스포츠용품을 제작·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G52">
@@ -4149,7 +4149,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국에서 푸시 알림·메신저·분석·문자·원클릭 인증 등 개발자 서비스와 산업별 앱을 제공하는 기업.</ns0:t>
+          <ns0:t>중국에서 푸시 알림·메신저·분석·문자·원클릭 인증 등 개발자 서비스와 산업별 앱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4228,7 +4228,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>소셜 서비스와 통신 기술을 제공하며 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영한다.</ns0:t>
+          <ns0:t>소셜 서비스·통신 기술을 제공하고 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4386,7 +4386,7 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>치료제를 개발·상용화하는 바이오제약사로, 재발성 심낭염 치료제 ARCALYST를 제공.</ns0:t>
+          <ns0:t>치료제를 개발·상용화하며 재발성 심낭염 치료제 ARCALYST를 제공하는 바이오제약사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56">
@@ -4465,7 +4465,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>탄산음료·생수·스포츠음료·커피·차·주스·유제품·식물성 음료 등 비알코올 음료를 제조·판매.</ns0:t>
+          <ns0:t>탄산음료·생수·스포츠음료·커피·차·주스·유제품·식물성 음료 등 비알코올 음료 제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4623,7 +4623,7 @@
       </ns0:c>
       <ns0:c r="F59" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득하는 기업.</ns0:t>
+          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G59">
@@ -4702,7 +4702,7 @@
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>고령자 주거시설과 의료시설에 임대·합작투자·구조화 금융 등으로 투자하는 부동산투자신탁.</ns0:t>
+          <ns0:t>고령자 주거·의료시설에 임대·합작투자·구조화 금융 등으로 투자하는 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60">
@@ -4781,7 +4781,7 @@
       </ns0:c>
       <ns0:c r="F61" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 거래 처리 및 결제 관련 제품·서비스를 소비자, 가맹점, 금융기관 등에 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소비자·가맹점·금융기관 등에 거래 처리와 결제 제품·서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G61">
@@ -4860,7 +4860,7 @@
       </ns0:c>
       <ns0:c r="F62" t="inlineStr">
         <ns0:is>
-          <ns0:t>공급망·재고·옴니채널 운영과 창고 관리를 위한 소프트웨어를 개발·판매·구축·유지보수.</ns0:t>
+          <ns0:t>공급망·재고·옴니채널 운영·창고 관리 소프트웨어를 개발·판매·구축·유지보수하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G62">
@@ -4939,7 +4939,7 @@
       </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
-          <ns0:t>의약품 유통, 종양·전문진료, 처방 기술, 의료·외과용품 관련 의료 서비스를 제공.</ns0:t>
+          <ns0:t>의약품 유통·종양 및 전문진료·처방 기술·의료 및 외과용품 관련 의료 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G63">
@@ -5097,7 +5097,7 @@
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통한다.</ns0:t>
+          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65">
@@ -5176,7 +5176,7 @@
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66">
@@ -5255,7 +5255,7 @@
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67">
@@ -5334,7 +5334,7 @@
       </ns0:c>
       <ns0:c r="F68" t="inlineStr">
         <ns0:is>
-          <ns0:t>자동차 금융·리스, 은행 및 금융서비스 산업용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
+          <ns0:t>자동차 금융·리스, 은행·금융서비스용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G68">
@@ -5413,7 +5413,7 @@
       </ns0:c>
       <ns0:c r="F69" t="inlineStr">
         <ns0:is>
-          <ns0:t>가정·상업·산업 고객에게 전력과 천연가스를 생산·구매·운송·공급하는 에너지 기업.</ns0:t>
+          <ns0:t>가정·상업·산업 고객에게 전력·천연가스를 생산·구매·운송·공급하는 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G69">
@@ -5492,7 +5492,7 @@
       </ns0:c>
       <ns0:c r="F70" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 중소·중견기업에 채용 등 고용 전 과정을 관리하는 클라우드 인적자본관리 소프트웨어를 제공.</ns0:t>
+          <ns0:t>미국 중소·중견기업에 채용 등 고용 전 과정을 관리하는 클라우드 인적자본관리 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G70">
@@ -5571,7 +5571,7 @@
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>선불카드, 환자 비용 부담 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
+          <ns0:t>선불카드, 환자 비용 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71">
@@ -5650,7 +5650,7 @@
       </ns0:c>
       <ns0:c r="F72" t="inlineStr">
         <ns0:is>
-          <ns0:t>암 치료 제품을 개발·상용화하는 바이오제약 기업으로 경구용 네라티닙인 NERLYNX를 제공.</ns0:t>
+          <ns0:t>암 치료제를 개발·상용화하는 바이오제약 기업으로 경구용 네라티닙 NERLYNX 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G72">
@@ -5729,7 +5729,7 @@
       </ns0:c>
       <ns0:c r="F73" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료진 대상 비마약성 통증관리·재생건강 솔루션을 개발·제조·판매하며 수술 후 통증관리 주사제를 제공.</ns0:t>
+          <ns0:t>비마약성 통증관리·재생건강 솔루션과 수술 후 통증관리 주사제를 개발·제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G73">
@@ -5808,7 +5808,7 @@
       </ns0:c>
       <ns0:c r="F74" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 급여·세무·인사 관리 등을 지원하는 클라우드 인적자본관리·재무·IT 소프트웨어를 제공.</ns0:t>
+          <ns0:t>미국에서 급여·세무·인사 관리를 지원하는 클라우드 인적자본관리·재무·IT 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G74">
@@ -5887,7 +5887,7 @@
       </ns0:c>
       <ns0:c r="F75" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 바이오의약품을 발굴·개발·제조·마케팅·유통·판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 바이오의약품을 발굴·개발·제조·마케팅·유통·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G75">
@@ -5966,7 +5966,7 @@
       </ns0:c>
       <ns0:c r="F76" t="inlineStr">
         <ns0:is>
-          <ns0:t>담배와 IQOS·VEEV·ZYN 브랜드의 가열담배·전자담배·경구용 니코틴 제품 및 액세서리를 판매.</ns0:t>
+          <ns0:t>담배와 IQOS·VEEV·ZYN 브랜드의 가열담배·전자담배·경구용 니코틴 제품 및 액세서리 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G76">
@@ -6045,7 +6045,7 @@
       </ns0:c>
       <ns0:c r="F77" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 교육 교재·평가·자격인증·온라인 학습·영어 학습 등 교육 서비스를 제공.</ns0:t>
+          <ns0:t>세계 각지에서 교육 교재·평가·자격인증·온라인 학습·영어 학습 등 교육 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G77">
@@ -6124,7 +6124,7 @@
       </ns0:c>
       <ns0:c r="F78" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 생명·건강 및 자산집약형 재보험을 제공하며 장애·장기요양 관련 보장도 취급.</ns0:t>
+          <ns0:t>전 세계에서 생명·건강·자산집약형 재보험을 제공하고 장애·장기요양 관련 보장도 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G78">
@@ -6203,7 +6203,7 @@
       </ns0:c>
       <ns0:c r="F79" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 재산·상해·특종 보험과 재보험을 제공하며 재산 재해 초과손해 재보험을 취급.</ns0:t>
+          <ns0:t>미국과 해외에서 재산·상해·특종 보험 및 재보험을 제공하고 재산 재해 초과손해 재보험 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G79">
@@ -6361,7 +6361,7 @@
       </ns0:c>
       <ns0:c r="F81" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 건강한 음식과 음료를 제공하는 패스트푸드 식당을 운영하며 온라인·모바일 주문을 지원.</ns0:t>
+          <ns0:t>미국에서 건강한 음식·음료를 제공하는 패스트푸드 식당을 운영하고 온라인·모바일 주문 지원.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G81">
@@ -6440,7 +6440,7 @@
       </ns0:c>
       <ns0:c r="F82" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국·아일랜드에서 다이아몬드 주얼리 소매점을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국·아일랜드에서 다이아몬드 주얼리 소매점을 운영하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G82">
@@ -6519,7 +6519,7 @@
       </ns0:c>
       <ns0:c r="F83" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의사·병원·클리닉·급성기 이후 치료시설에 수술용 의료 솔루션을 개발·판매·유통.</ns0:t>
+          <ns0:t>미국 의사·병원·클리닉·급성기 이후 치료시설 대상 수술용 의료 솔루션 개발·판매·유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G83">
@@ -6598,7 +6598,7 @@
       </ns0:c>
       <ns0:c r="F84" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·중국 및 해외에서 유무선·핸디형·로봇 청소기 등 소비자용 제품을 설계·제공.</ns0:t>
+          <ns0:t>미국·중국 및 해외에서 유무선·핸디형·로봇 청소기 등 소비자용 제품을 설계·제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G84">
@@ -6677,7 +6677,7 @@
       </ns0:c>
       <ns0:c r="F85" t="inlineStr">
         <ns0:is>
-          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청, 연료, 나프타, 윤활유, 액화석유가스 등을 공급한다.</ns0:t>
+          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청·연료·나프타·윤활유·액화석유가스를 공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G85">
@@ -6756,7 +6756,7 @@
       </ns0:c>
       <ns0:c r="F86" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 영위하는 종합 에너지 기업.</ns0:t>
+          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 운영하는 종합 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G86">
@@ -6835,7 +6835,7 @@
       </ns0:c>
       <ns0:c r="F87" t="inlineStr">
         <ns0:is>
-          <ns0:t>소화기·희귀질환·혈장유래 치료·종양·백신·신경과학 분야 의약품을 연구·개발·제조·판매·기술이전.</ns0:t>
+          <ns0:t>소화기·희귀질환·혈장유래 치료·종양·백신·신경과학 분야 의약품 연구·개발·제조·판매·기술이전.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G87">
@@ -7072,7 +7072,7 @@
       </ns0:c>
       <ns0:c r="F90" t="inlineStr">
         <ns0:is>
-          <ns0:t>실질적인 영업활동 없이 다른 기업과의 합병·주식교환·자산인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>실질적 영업활동 없이 합병·주식교환·자산인수 등 다른 기업과의 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G90">
@@ -7148,7 +7148,7 @@
       </ns0:c>
       <ns0:c r="F91" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 소매·도매·구독 사업으로 의류·신발·액세서리 등 라이프스타일 상품과 서비스 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소매·도매·구독 사업을 통해 의류·신발·액세서리 등 라이프스타일 상품·서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G91">
@@ -7227,7 +7227,7 @@
       </ns0:c>
       <ns0:c r="F92" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 감자칩·토르티야칩·프레첼·치즈 스낵·돼지껍질·팝콘 등 브랜드 짭짤한 간식을 제조.</ns0:t>
+          <ns0:t>미국에서 감자칩·토르티야칩·프레첼·치즈 스낵·돼지껍질·팝콘 등 브랜드 짭짤한 간식 제조.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G92">
@@ -7385,7 +7385,7 @@
       </ns0:c>
       <ns0:c r="F94" t="inlineStr">
         <ns0:is>
-          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공.</ns0:t>
+          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G94">
@@ -7464,7 +7464,7 @@
       </ns0:c>
       <ns0:c r="F95" t="inlineStr">
         <ns0:is>
-          <ns0:t>버지니아 내 상업·개인 금융 서비스를 제공하는 은행의 지주회사로 은행 및 신탁·상속재산 서비스 운영.</ns0:t>
+          <ns0:t>버지니아에서 상업·개인 금융과 신탁·상속재산 서비스를 운영하는 은행 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G95">
@@ -7543,7 +7543,7 @@
       </ns0:c>
       <ns0:c r="F96" t="inlineStr">
         <ns0:is>
-          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 이동통신과 디지털 서비스를 제공.</ns0:t>
+          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 이동통신·디지털 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G96">

</xml_diff>